<commit_message>
feat(config): 完善 Luban 基础表与可读 ID
背景：基础数据表需要采用策划可识别的中文文件名、人工可读 ID，并补充游戏全局常量入口。

变更内容：统一业务工作簿为拼音首字母_中文_英文命名；全部工作表有效区域改为水平和垂直居中；删除未被运行时代码使用且与 id 重复的 key 字段；补充源表保护、命名和 ID 规范。

数据表与生成物：新增 GameConfig，包含初始角色、初始解锁角色、初始解锁技能和首关引用；资源 ID 使用 CTNNNN，动画和表现集合使用 CNNNN，角色与怪物从 10001 起，技能沿用 20000+资源编号；既有 ID 保持不变；重新生成全部相关 C# 类型和 bytes。

验证：Tools/Config/generate.ps1 通过；Git Bash 执行 Tools/Config/generate.sh 通过；dotnet build Roguelike.slnx 结果为 0 警告、0 错误；15 张工作簿逐表校验 key 已移除、ID 未变化、有效单元格全部居中。

影响与风险：配置二进制结构因移除 key 而变化，运行时必须与本次生成代码配套使用；当前手写代码未使用 Key，未发现兼容风险。

未包含：不包含 MCPDemo 场景改动；不包含临时 ConfigService 及后续模块架构重构。
</commit_message>
<xml_diff>
--- a/Config/Datas/__beans__.xlsx
+++ b/Config/Datas/__beans__.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Beans" sheetId="1" r:id="R40b3e681df024f88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Beans" sheetId="1" r:id="R0ee372acb99e415e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -159,95 +159,98 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="31">
+  <x:cellXfs count="32">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
+      <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -470,144 +473,144 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="24" t="str">
+      <x:c r="A1" s="25" t="str">
         <x:v>##var</x:v>
       </x:c>
-      <x:c r="B1" s="9" t="str">
+      <x:c r="B1" s="10" t="str">
         <x:v>full_name</x:v>
       </x:c>
-      <x:c r="C1" s="9" t="str">
+      <x:c r="C1" s="10" t="str">
         <x:v>parent</x:v>
       </x:c>
-      <x:c r="D1" s="9" t="str">
+      <x:c r="D1" s="10" t="str">
         <x:v>valueType</x:v>
       </x:c>
-      <x:c r="E1" s="9" t="str">
+      <x:c r="E1" s="10" t="str">
         <x:v>alias</x:v>
       </x:c>
-      <x:c r="F1" s="9" t="str">
+      <x:c r="F1" s="10" t="str">
         <x:v>sep</x:v>
       </x:c>
-      <x:c r="G1" s="9" t="str">
+      <x:c r="G1" s="10" t="str">
         <x:v>comment</x:v>
       </x:c>
-      <x:c r="H1" s="9" t="str">
+      <x:c r="H1" s="10" t="str">
         <x:v>tags</x:v>
       </x:c>
-      <x:c r="I1" s="9" t="str">
+      <x:c r="I1" s="10" t="str">
         <x:v>group</x:v>
       </x:c>
-      <x:c r="J1" s="9" t="str">
+      <x:c r="J1" s="10" t="str">
         <x:v>*fields</x:v>
       </x:c>
-      <x:c r="K1" s="9"/>
-      <x:c r="L1" s="9"/>
-      <x:c r="M1" s="9"/>
-      <x:c r="N1" s="9"/>
-      <x:c r="O1" s="9"/>
-      <x:c r="P1" s="10"/>
+      <x:c r="K1" s="10"/>
+      <x:c r="L1" s="10"/>
+      <x:c r="M1" s="10"/>
+      <x:c r="N1" s="10"/>
+      <x:c r="O1" s="10"/>
+      <x:c r="P1" s="11"/>
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
-      <x:c r="A2" s="28" t="str">
+      <x:c r="A2" s="29" t="str">
         <x:v>##var</x:v>
       </x:c>
-      <x:c r="B2" s="13"/>
-      <x:c r="C2" s="13"/>
-      <x:c r="D2" s="13"/>
-      <x:c r="E2" s="13"/>
-      <x:c r="F2" s="13"/>
-      <x:c r="G2" s="13"/>
-      <x:c r="H2" s="13"/>
-      <x:c r="I2" s="13"/>
-      <x:c r="J2" s="13" t="str">
+      <x:c r="B2" s="14"/>
+      <x:c r="C2" s="14"/>
+      <x:c r="D2" s="14"/>
+      <x:c r="E2" s="14"/>
+      <x:c r="F2" s="14"/>
+      <x:c r="G2" s="14"/>
+      <x:c r="H2" s="14"/>
+      <x:c r="I2" s="14"/>
+      <x:c r="J2" s="14" t="str">
         <x:v>name</x:v>
       </x:c>
-      <x:c r="K2" s="13" t="str">
+      <x:c r="K2" s="14" t="str">
         <x:v>alias</x:v>
       </x:c>
-      <x:c r="L2" s="13" t="str">
+      <x:c r="L2" s="14" t="str">
         <x:v>type</x:v>
       </x:c>
-      <x:c r="M2" s="13" t="str">
+      <x:c r="M2" s="14" t="str">
         <x:v>group</x:v>
       </x:c>
-      <x:c r="N2" s="13" t="str">
+      <x:c r="N2" s="14" t="str">
         <x:v>comment</x:v>
       </x:c>
-      <x:c r="O2" s="13" t="str">
+      <x:c r="O2" s="14" t="str">
         <x:v>tags</x:v>
       </x:c>
-      <x:c r="P2" s="13" t="str">
+      <x:c r="P2" s="14" t="str">
         <x:v>variants</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="30" customHeight="1">
-      <x:c r="A3" s="29" t="str">
+      <x:c r="A3" s="30" t="str">
         <x:v>##</x:v>
       </x:c>
-      <x:c r="B3" s="15" t="str">
+      <x:c r="B3" s="16" t="str">
         <x:v>完整类型名</x:v>
       </x:c>
-      <x:c r="C3" s="15" t="str">
+      <x:c r="C3" s="16" t="str">
         <x:v>父类型</x:v>
       </x:c>
-      <x:c r="D3" s="15" t="str">
+      <x:c r="D3" s="16" t="str">
         <x:v>值类型</x:v>
       </x:c>
-      <x:c r="E3" s="15" t="str">
+      <x:c r="E3" s="16" t="str">
         <x:v>别名</x:v>
       </x:c>
-      <x:c r="F3" s="15" t="str">
+      <x:c r="F3" s="16" t="str">
         <x:v>分隔符</x:v>
       </x:c>
-      <x:c r="G3" s="15" t="str">
+      <x:c r="G3" s="16" t="str">
         <x:v>说明</x:v>
       </x:c>
-      <x:c r="H3" s="15" t="str">
+      <x:c r="H3" s="16" t="str">
         <x:v>标签</x:v>
       </x:c>
-      <x:c r="I3" s="15" t="str">
+      <x:c r="I3" s="16" t="str">
         <x:v>分组</x:v>
       </x:c>
-      <x:c r="J3" s="15" t="str">
+      <x:c r="J3" s="16" t="str">
         <x:v>字段名</x:v>
       </x:c>
-      <x:c r="K3" s="15" t="str">
+      <x:c r="K3" s="16" t="str">
         <x:v>别名</x:v>
       </x:c>
-      <x:c r="L3" s="15" t="str">
+      <x:c r="L3" s="16" t="str">
         <x:v>字段类型</x:v>
       </x:c>
-      <x:c r="M3" s="15" t="str">
+      <x:c r="M3" s="16" t="str">
         <x:v>分组</x:v>
       </x:c>
-      <x:c r="N3" s="15" t="str">
+      <x:c r="N3" s="16" t="str">
         <x:v>说明</x:v>
       </x:c>
-      <x:c r="O3" s="15" t="str">
+      <x:c r="O3" s="16" t="str">
         <x:v>标签</x:v>
       </x:c>
-      <x:c r="P3" s="15" t="str">
+      <x:c r="P3" s="16" t="str">
         <x:v>变体</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
-      <x:c r="A4" s="30"/>
-      <x:c r="B4" s="22"/>
-      <x:c r="C4" s="22"/>
-      <x:c r="D4" s="22"/>
-      <x:c r="E4" s="22"/>
-      <x:c r="F4" s="22"/>
-      <x:c r="G4" s="22"/>
-      <x:c r="H4" s="22"/>
-      <x:c r="I4" s="22"/>
-      <x:c r="J4" s="22"/>
-      <x:c r="K4" s="22"/>
-      <x:c r="L4" s="22"/>
-      <x:c r="M4" s="22"/>
-      <x:c r="N4" s="22"/>
-      <x:c r="O4" s="22"/>
-      <x:c r="P4" s="23"/>
+      <x:c r="A4" s="31"/>
+      <x:c r="B4" s="23"/>
+      <x:c r="C4" s="23"/>
+      <x:c r="D4" s="23"/>
+      <x:c r="E4" s="23"/>
+      <x:c r="F4" s="23"/>
+      <x:c r="G4" s="23"/>
+      <x:c r="H4" s="23"/>
+      <x:c r="I4" s="23"/>
+      <x:c r="J4" s="23"/>
+      <x:c r="K4" s="23"/>
+      <x:c r="L4" s="23"/>
+      <x:c r="M4" s="23"/>
+      <x:c r="N4" s="23"/>
+      <x:c r="O4" s="23"/>
+      <x:c r="P4" s="24"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>